<commit_message>
Add API endpoint for Abril photos loading
- Created /api/agrosuper/abril-photos endpoint
- Fetches photos from agrosuper_abril_photos table by form_code
- Groups photos by type (bandeja_jamon_lc, logo_vitrina_lc, etc.)
- Returns organized JSON structure for frontend display
- Fixes "no photos available" issue in Abril campaign

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Agrosuper Abril.xlsx
+++ b/Agrosuper Abril.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berni\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berni\Documentos\Pag Agrosuper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6E8F4B7-9A07-4268-A6E1-9687D671FBDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4390F8EC-6B9E-41B1-A1C2-EDC280A9905A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6554,9 +6554,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Arial"/>
       <family val="1"/>
     </font>
@@ -6578,13 +6585,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -7451,7 +7461,7 @@
       <c r="P3" t="s">
         <v>72</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R3" t="s">
@@ -42804,6 +42814,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="Q3" r:id="rId1" xr:uid="{90E1C178-3D35-4EA5-9B31-FC222CDD55EE}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>